<commit_message>
adjusting BC importation to retrieve data automaticaly
</commit_message>
<xml_diff>
--- a/BC.xlsx
+++ b/BC.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dell\Desktop\antiGravity\estf-magasiner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{015B1EF1-8D10-4EA1-8988-759A717D541E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BC67E1A-47FA-46DE-8556-A4E04DCBA30F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -27,9 +27,10 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -479,25 +480,213 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" readingOrder="2"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -506,18 +695,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -526,182 +703,6 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="7" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1627,204 +1628,204 @@
       <c r="C7" s="1"/>
     </row>
     <row r="9" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="72" t="s">
         <v>23</v>
       </c>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
+      <c r="B9" s="72"/>
+      <c r="C9" s="72"/>
+      <c r="D9" s="72"/>
+      <c r="E9" s="72"/>
+      <c r="F9" s="72"/>
+      <c r="G9" s="72"/>
+      <c r="H9" s="72"/>
     </row>
     <row r="10" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
+      <c r="A10" s="4"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="4"/>
     </row>
     <row r="11" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="73" t="s">
         <v>0</v>
       </c>
-      <c r="B11" s="6"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="8" t="s">
+      <c r="B11" s="73"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="74" t="s">
         <v>1</v>
       </c>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="9"/>
+      <c r="E11" s="74"/>
+      <c r="F11" s="74"/>
+      <c r="G11" s="6"/>
       <c r="H11" s="1"/>
     </row>
     <row r="12" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A12" s="10"/>
-      <c r="B12" s="10"/>
-      <c r="C12" s="11" t="s">
+      <c r="A12" s="7"/>
+      <c r="B12" s="7"/>
+      <c r="C12" s="75" t="s">
         <v>24</v>
       </c>
-      <c r="D12" s="11"/>
-      <c r="E12" s="11"/>
-      <c r="F12" s="11"/>
-      <c r="G12" s="11"/>
-      <c r="H12" s="11"/>
+      <c r="D12" s="75"/>
+      <c r="E12" s="75"/>
+      <c r="F12" s="75"/>
+      <c r="G12" s="75"/>
+      <c r="H12" s="75"/>
     </row>
     <row r="13" spans="1:10" ht="13.5" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="14" spans="1:10" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="12" t="s">
+      <c r="A14" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B14" s="12" t="s">
+      <c r="B14" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="C14" s="12" t="s">
+      <c r="C14" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="D14" s="13" t="s">
+      <c r="D14" s="76" t="s">
         <v>4</v>
       </c>
-      <c r="E14" s="13"/>
-      <c r="F14" s="13"/>
-      <c r="G14" s="12" t="s">
+      <c r="E14" s="76"/>
+      <c r="F14" s="76"/>
+      <c r="G14" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="H14" s="14" t="s">
+      <c r="H14" s="9" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="12">
+      <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="15">
+      <c r="B15" s="10">
         <v>1</v>
       </c>
-      <c r="C15" s="16" t="s">
+      <c r="C15" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="D15" s="17" t="s">
+      <c r="D15" s="77" t="s">
         <v>22</v>
       </c>
-      <c r="E15" s="18"/>
-      <c r="F15" s="19"/>
-      <c r="G15" s="20"/>
-      <c r="H15" s="21">
+      <c r="E15" s="78"/>
+      <c r="F15" s="79"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="13">
         <f>+G15*B15</f>
         <v>0</v>
       </c>
-      <c r="I15" s="22"/>
-      <c r="J15" s="22"/>
+      <c r="I15" s="14"/>
+      <c r="J15" s="14"/>
     </row>
     <row r="16" spans="1:10" ht="13.5" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="23">
+      <c r="A16" s="58">
         <v>2</v>
       </c>
-      <c r="B16" s="24">
+      <c r="B16" s="60">
         <v>2</v>
       </c>
-      <c r="C16" s="24" t="s">
+      <c r="C16" s="60" t="s">
         <v>21</v>
       </c>
-      <c r="D16" s="25" t="s">
+      <c r="D16" s="62" t="s">
         <v>25</v>
       </c>
-      <c r="E16" s="26"/>
-      <c r="F16" s="27"/>
-      <c r="G16" s="28"/>
-      <c r="H16" s="29">
+      <c r="E16" s="63"/>
+      <c r="F16" s="64"/>
+      <c r="G16" s="68"/>
+      <c r="H16" s="70">
         <f>+G16*B16</f>
         <v>0</v>
       </c>
-      <c r="I16" s="22"/>
-      <c r="J16" s="22"/>
+      <c r="I16" s="14"/>
+      <c r="J16" s="14"/>
     </row>
     <row r="17" spans="1:10" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="30"/>
-      <c r="B17" s="31"/>
-      <c r="C17" s="31"/>
-      <c r="D17" s="32"/>
-      <c r="E17" s="33"/>
-      <c r="F17" s="34"/>
-      <c r="G17" s="35"/>
-      <c r="H17" s="36"/>
-      <c r="I17" s="22"/>
-      <c r="J17" s="22"/>
+      <c r="A17" s="59"/>
+      <c r="B17" s="61"/>
+      <c r="C17" s="61"/>
+      <c r="D17" s="65"/>
+      <c r="E17" s="66"/>
+      <c r="F17" s="67"/>
+      <c r="G17" s="69"/>
+      <c r="H17" s="71"/>
+      <c r="I17" s="14"/>
+      <c r="J17" s="14"/>
     </row>
     <row r="18" spans="1:10" ht="15.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="37" t="s">
+      <c r="A18" s="46" t="s">
         <v>7</v>
       </c>
-      <c r="B18" s="38"/>
-      <c r="C18" s="38"/>
-      <c r="D18" s="38"/>
-      <c r="E18" s="38"/>
-      <c r="F18" s="38"/>
-      <c r="G18" s="39"/>
-      <c r="H18" s="40">
+      <c r="B18" s="47"/>
+      <c r="C18" s="47"/>
+      <c r="D18" s="47"/>
+      <c r="E18" s="47"/>
+      <c r="F18" s="47"/>
+      <c r="G18" s="48"/>
+      <c r="H18" s="15">
         <f>SUM(H15:H17)</f>
         <v>0</v>
       </c>
-      <c r="I18" s="22"/>
-      <c r="J18" s="22"/>
+      <c r="I18" s="14"/>
+      <c r="J18" s="14"/>
     </row>
     <row r="19" spans="1:10" ht="15.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="37" t="s">
+      <c r="A19" s="46" t="s">
         <v>8</v>
       </c>
-      <c r="B19" s="38"/>
-      <c r="C19" s="38"/>
-      <c r="D19" s="38"/>
-      <c r="E19" s="38"/>
-      <c r="F19" s="38"/>
-      <c r="G19" s="39"/>
-      <c r="H19" s="41">
+      <c r="B19" s="47"/>
+      <c r="C19" s="47"/>
+      <c r="D19" s="47"/>
+      <c r="E19" s="47"/>
+      <c r="F19" s="47"/>
+      <c r="G19" s="48"/>
+      <c r="H19" s="16">
         <f>H18*20%</f>
         <v>0</v>
       </c>
-      <c r="I19" s="22"/>
-      <c r="J19" s="22"/>
+      <c r="I19" s="14"/>
+      <c r="J19" s="14"/>
     </row>
     <row r="20" spans="1:10" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="37" t="s">
+      <c r="A20" s="46" t="s">
         <v>9</v>
       </c>
-      <c r="B20" s="38"/>
-      <c r="C20" s="38"/>
-      <c r="D20" s="38"/>
-      <c r="E20" s="38"/>
-      <c r="F20" s="38"/>
-      <c r="G20" s="39"/>
-      <c r="H20" s="42">
+      <c r="B20" s="47"/>
+      <c r="C20" s="47"/>
+      <c r="D20" s="47"/>
+      <c r="E20" s="47"/>
+      <c r="F20" s="47"/>
+      <c r="G20" s="48"/>
+      <c r="H20" s="17">
         <f>H18+H19</f>
         <v>0</v>
       </c>
-      <c r="I20" s="43"/>
+      <c r="I20" s="18"/>
     </row>
     <row r="21" spans="1:10" ht="13.5" thickTop="1" x14ac:dyDescent="0.2"/>
     <row r="22" spans="1:10" ht="13.5" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="23" spans="1:10" ht="13.5" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="44" t="s">
+      <c r="A23" s="49" t="s">
         <v>10</v>
       </c>
-      <c r="B23" s="45"/>
-      <c r="C23" s="46"/>
-      <c r="D23" s="47"/>
-      <c r="E23" s="48"/>
-      <c r="F23" s="49" t="s">
+      <c r="B23" s="50"/>
+      <c r="C23" s="19"/>
+      <c r="D23" s="53"/>
+      <c r="E23" s="20"/>
+      <c r="F23" s="21" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="50"/>
-      <c r="B24" s="51"/>
-      <c r="C24" s="52"/>
-      <c r="D24" s="53"/>
-      <c r="E24" s="54"/>
-      <c r="F24" s="49" t="s">
+      <c r="A24" s="51"/>
+      <c r="B24" s="52"/>
+      <c r="C24" s="22"/>
+      <c r="D24" s="54"/>
+      <c r="E24" s="23"/>
+      <c r="F24" s="21" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1833,88 +1834,107 @@
         <v>13</v>
       </c>
       <c r="B25" s="56"/>
-      <c r="C25" s="57"/>
-      <c r="D25" s="58"/>
-      <c r="E25" s="48"/>
-      <c r="F25" s="59"/>
-      <c r="G25" s="59"/>
-      <c r="H25" s="59"/>
+      <c r="C25" s="24"/>
+      <c r="D25" s="25"/>
+      <c r="E25" s="20"/>
+      <c r="F25" s="57"/>
+      <c r="G25" s="57"/>
+      <c r="H25" s="57"/>
     </row>
     <row r="26" spans="1:10" ht="15.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="60" t="s">
+      <c r="A26" s="41" t="s">
         <v>14</v>
       </c>
-      <c r="B26" s="61"/>
-      <c r="C26" s="62"/>
-      <c r="D26" s="63"/>
-      <c r="E26" s="48"/>
-      <c r="F26" s="64"/>
-      <c r="G26" s="64"/>
-      <c r="H26" s="64"/>
+      <c r="B26" s="42"/>
+      <c r="C26" s="43"/>
+      <c r="D26" s="26"/>
+      <c r="E26" s="20"/>
+      <c r="F26" s="27"/>
+      <c r="G26" s="27"/>
+      <c r="H26" s="27"/>
     </row>
     <row r="27" spans="1:10" ht="13.5" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="65" t="s">
+      <c r="A27" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="B27" s="66"/>
-      <c r="C27" s="67"/>
-      <c r="D27" s="68"/>
-      <c r="E27" s="69"/>
-      <c r="F27" s="70"/>
-      <c r="G27" s="70"/>
-      <c r="H27" s="70"/>
+      <c r="B27" s="37"/>
+      <c r="C27" s="28"/>
+      <c r="D27" s="29"/>
+      <c r="E27" s="30"/>
+      <c r="F27" s="44"/>
+      <c r="G27" s="44"/>
+      <c r="H27" s="44"/>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A28" s="65" t="s">
+      <c r="A28" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="B28" s="66"/>
-      <c r="C28" s="67"/>
-      <c r="D28" s="71"/>
-      <c r="E28" s="72"/>
+      <c r="B28" s="37"/>
+      <c r="C28" s="28"/>
+      <c r="D28" s="31"/>
+      <c r="E28" s="32"/>
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
     </row>
     <row r="29" spans="1:10" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A29" s="65" t="s">
+      <c r="A29" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="B29" s="66"/>
-      <c r="C29" s="67"/>
-      <c r="D29" s="71"/>
-      <c r="E29" s="72"/>
-      <c r="F29" s="73" t="s">
+      <c r="B29" s="37"/>
+      <c r="C29" s="28"/>
+      <c r="D29" s="31"/>
+      <c r="E29" s="32"/>
+      <c r="F29" s="45" t="s">
         <v>26</v>
       </c>
-      <c r="G29" s="73"/>
-      <c r="H29" s="73"/>
+      <c r="G29" s="45"/>
+      <c r="H29" s="45"/>
     </row>
     <row r="30" spans="1:10" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="65" t="s">
+      <c r="A30" s="36" t="s">
         <v>18</v>
       </c>
-      <c r="B30" s="66"/>
-      <c r="C30" s="67"/>
-      <c r="D30" s="74"/>
+      <c r="B30" s="37"/>
+      <c r="C30" s="28"/>
+      <c r="D30" s="33"/>
     </row>
     <row r="31" spans="1:10" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="75" t="s">
+      <c r="A31" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="B31" s="76"/>
-      <c r="C31" s="77"/>
-      <c r="D31" s="78">
+      <c r="B31" s="39"/>
+      <c r="C31" s="34"/>
+      <c r="D31" s="35">
         <v>2024</v>
       </c>
-      <c r="F31" s="79" t="s">
+      <c r="F31" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="G31" s="79"/>
+      <c r="G31" s="40"/>
     </row>
     <row r="32" spans="1:10" ht="13.5" thickTop="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="28">
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="C12:H12"/>
+    <mergeCell ref="D14:F14"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="F25:H25"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="D16:F17"/>
+    <mergeCell ref="G16:G17"/>
+    <mergeCell ref="H16:H17"/>
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A19:G19"/>
+    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="A23:B24"/>
+    <mergeCell ref="D23:D24"/>
     <mergeCell ref="A30:B30"/>
     <mergeCell ref="A31:B31"/>
     <mergeCell ref="F31:G31"/>
@@ -1924,25 +1944,6 @@
     <mergeCell ref="A28:B28"/>
     <mergeCell ref="A29:B29"/>
     <mergeCell ref="F29:H29"/>
-    <mergeCell ref="A18:G18"/>
-    <mergeCell ref="A19:G19"/>
-    <mergeCell ref="A20:G20"/>
-    <mergeCell ref="A23:B24"/>
-    <mergeCell ref="D23:D24"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="F25:H25"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="D16:F17"/>
-    <mergeCell ref="G16:G17"/>
-    <mergeCell ref="H16:H17"/>
-    <mergeCell ref="A9:H9"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="C12:H12"/>
-    <mergeCell ref="D14:F14"/>
-    <mergeCell ref="D15:F15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>